<commit_message>
Final QA pass: content gaps, formatting, and PDF print fixes
Content fixes:
- 11-filled-example.docx: now has 5 tables (physical supply, monetary
  supply, physical use, monetary use, integrated SUT)
- Exercise workbook README: added Step 7 (SUT) explanation
- Answers sheet: SUT answers included

Formatting QA:
- Ran format_qa.py on all 51 Word docs across all 8 notebooks
- Checked for: ** markdown artifacts, orphaned titles, table widths,
  consecutive blanks, font consistency
- Result: 51 files checked, 0 issues found (clean)

PDF print fixes:
- Injected @media print CSS into all 21 HTML visual slides:
  @page { size: A4 landscape; margin: 10mm }
  Content scales to fit, no cutoff, shadows removed for print
- Regenerated all 16 PDFs with Chrome headless
- Updated all notebook PDF copies

All print-notebooks/03-services/ files now verified:
  Supply: all 15 files YES
  Use: all 15 files YES
  SUT: all 15 files YES

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/s-s-event-bogor/print-notebooks/03-services/11-exercise-workbook.xlsx
+++ b/s-s-event-bogor/print-notebooks/03-services/11-exercise-workbook.xlsx
@@ -935,7 +935,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A26"/>
+  <dimension ref="A1:A33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="90" customWidth="1" min="1" max="1"/>
@@ -1068,6 +1068,48 @@
       <c r="A26" s="6" t="inlineStr">
         <is>
           <t xml:space="preserve">  - The use table total must match the supply table total</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Step 7: Build the integrated Supply-Use Table (SEEA EA Table 7.1)</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  - Combines supply and use in one table</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  - SUPPLY half: fill ecosystem columns (where services come from)</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  - USE half: fill economic unit columns (who benefits)</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  - Check: Total supply = Total use for each service row</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  - This is the standard SEEA EA output format</t>
         </is>
       </c>
     </row>
@@ -3392,6 +3434,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="4" t="inlineStr">
         <is>
@@ -3399,6 +3442,7 @@
         </is>
       </c>
     </row>
+    <row r="4"/>
     <row r="5">
       <c r="A5" s="11" t="inlineStr">
         <is>
@@ -3406,6 +3450,7 @@
         </is>
       </c>
     </row>
+    <row r="6"/>
     <row r="7">
       <c r="A7" s="7" t="inlineStr">
         <is>
@@ -3560,6 +3605,8 @@
         </is>
       </c>
     </row>
+    <row r="14"/>
+    <row r="15"/>
     <row r="16">
       <c r="A16" s="11" t="inlineStr">
         <is>
@@ -3567,6 +3614,7 @@
         </is>
       </c>
     </row>
+    <row r="17"/>
     <row r="18">
       <c r="A18" s="7" t="inlineStr">
         <is>
@@ -3695,6 +3743,8 @@
         <v>17400</v>
       </c>
     </row>
+    <row r="23"/>
+    <row r="24"/>
     <row r="25">
       <c r="A25" s="11" t="inlineStr">
         <is>
@@ -3702,6 +3752,7 @@
         </is>
       </c>
     </row>
+    <row r="26"/>
     <row r="27">
       <c r="A27" s="7" t="inlineStr">
         <is>
@@ -3787,6 +3838,8 @@
         </is>
       </c>
     </row>
+    <row r="32"/>
+    <row r="33"/>
     <row r="34">
       <c r="A34" s="11" t="inlineStr">
         <is>
@@ -3794,6 +3847,7 @@
         </is>
       </c>
     </row>
+    <row r="35"/>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
@@ -3846,6 +3900,7 @@
         <v>210000</v>
       </c>
     </row>
+    <row r="40"/>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
         <is>
@@ -3909,6 +3964,7 @@
         <v>119085</v>
       </c>
     </row>
+    <row r="45"/>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
@@ -3961,6 +4017,7 @@
         <v>1550000</v>
       </c>
     </row>
+    <row r="50"/>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
         <is>
@@ -4009,6 +4066,8 @@
         <v>1359000</v>
       </c>
     </row>
+    <row r="55"/>
+    <row r="56"/>
     <row r="57">
       <c r="A57" s="11" t="inlineStr">
         <is>
@@ -4016,6 +4075,7 @@
         </is>
       </c>
     </row>
+    <row r="58"/>
     <row r="59">
       <c r="A59" s="7" t="inlineStr">
         <is>
@@ -4164,6 +4224,7 @@
         <v>3238085</v>
       </c>
     </row>
+    <row r="65"/>
     <row r="66">
       <c r="A66" s="11" t="inlineStr">
         <is>
@@ -4171,6 +4232,7 @@
         </is>
       </c>
     </row>
+    <row r="67"/>
     <row r="68">
       <c r="A68" s="19" t="inlineStr">
         <is>
@@ -4235,6 +4297,7 @@
       <c r="E71" s="20" t="n"/>
       <c r="F71" s="21" t="n"/>
     </row>
+    <row r="72"/>
     <row r="73">
       <c r="A73" s="40" t="inlineStr">
         <is>
@@ -4242,6 +4305,7 @@
         </is>
       </c>
     </row>
+    <row r="74"/>
     <row r="75">
       <c r="A75" s="5" t="inlineStr">
         <is>
@@ -4291,6 +4355,7 @@
         </is>
       </c>
     </row>
+    <row r="82"/>
     <row r="83">
       <c r="A83" s="5" t="inlineStr">
         <is>
@@ -4520,6 +4585,7 @@
         <v>18000</v>
       </c>
     </row>
+    <row r="91"/>
     <row r="92">
       <c r="A92" s="5" t="inlineStr">
         <is>
@@ -4775,6 +4841,7 @@
         <v>3253835</v>
       </c>
     </row>
+    <row r="101"/>
     <row r="102">
       <c r="A102" s="5" t="inlineStr">
         <is>
@@ -4789,6 +4856,7 @@
         </is>
       </c>
     </row>
+    <row r="104"/>
     <row r="105">
       <c r="A105" s="45" t="inlineStr">
         <is>
@@ -4796,6 +4864,8 @@
         </is>
       </c>
     </row>
+    <row r="106"/>
+    <row r="107"/>
     <row r="108">
       <c r="A108" s="40" t="inlineStr">
         <is>
@@ -4803,6 +4873,7 @@
         </is>
       </c>
     </row>
+    <row r="109"/>
     <row r="110">
       <c r="A110" s="47" t="inlineStr">
         <is>
@@ -5124,6 +5195,7 @@
         <v>18000</v>
       </c>
     </row>
+    <row r="118"/>
     <row r="119">
       <c r="A119" s="47" t="inlineStr">
         <is>
@@ -5487,6 +5559,7 @@
         <v>3253835</v>
       </c>
     </row>
+    <row r="128"/>
     <row r="129">
       <c r="A129" s="50" t="inlineStr">
         <is>

</xml_diff>